<commit_message>
Ganti foto gel dengan foto pemilik + nama general, tambah aksi updateProductMeta
AB-G001 jadi 'Energy Gel' dan AB-G002 'Energy Gel Plus' tanpa klaim rasa/berat. Foto dipotong 3:4 dan dikompres (84 KB & 66 KB). Aksi GAS updateProductMeta mengubah nama/deskripsi/imageUrl tanpa membuka spreadsheet dan menginvalidasi cache produk.
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -978,7 +978,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Energy Gel Jeruk 30 g</t>
+          <t>Energy Gel</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Gel energi 30 g dengan 22 g karbohidrat, rasa jeruk. Dimakan 15–20 menit sebelum atau saat lari jauh.</t>
+          <t>Gel energi praktis dalam sachet sekali pakai. Cocok diminum 15–20 menit sebelum atau saat lari jauh.</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
@@ -996,7 +996,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>/products/ab-g001.svg</t>
+          <t>/products/ab-g001.jpg</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Energy Gel Kopi 30 g</t>
+          <t>Energy Gel Plus</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Gel energi rasa kopi dengan kafein 40 mg per sachet. Untuk sesi panjang atau lari pagi.</t>
+          <t>Gel energi dengan formula lebih pekat untuk sesi panjang. Praktis dibawa di kantong lari.</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>/products/ab-g002.svg</t>
+          <t>/products/ab-g002.jpg</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Tambah produk jam lari GPS dan kategori Jam
Tambah AB-J001 Jam Lari GPS Pace ke data demo, navbar, beranda, footer, dan katalog. Perbarui data/products.xlsx dan panduan spreadsheet untuk 11 produk.
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1120,6 +1120,56 @@
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="2" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AB-J001</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Jam Lari GPS Pace</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Jam</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Jam lari GPS dengan detak jantung pergelangan, pace dan rute real-time, serta baterai tahan hingga 14 hari. Ringan untuk sesi harian sampai lari jarak jauh.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1899000</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>/products/ab-j001.jpg</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>one</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="S12" s="2" t="n"/>
+      <c r="T12" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>